<commit_message>
ETA: Neues Wort aus Issue #5
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fortschritt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fortschritt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5415,6 +5415,62 @@
       <c r="L85" s="5" t="inlineStr">
         <is>
           <t>Kitchen/Cooking</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>napkin</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Serviette</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>/ˈnæpkɪn/</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>A piece of cloth or paper used to wipe mouth and hands while eating.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>She wiped her mouth with a napkin after dinner.</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Please put a napkin on your lap before eating.</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/Special:FilePath/Brede-LilleBrede-napkin.jpg?width=400</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>1</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #6
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5467,8 +5467,59 @@
           <t>2026-04-19</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>to struggle</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>kämpfen</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>/ˈstrʌɡəl/</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>To try very hard to do something difficult or to deal with a problem.</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>She struggled to open the heavy door.</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Many students struggle with mathematics.</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="n">
+        <v>2</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #7
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5509,7 +5509,6 @@
           <t>Many students struggle with mathematics.</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
       <c r="I87" t="n">
         <v>2</v>
       </c>
@@ -5518,8 +5517,63 @@
           <t>2026-04-19</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Democracy</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Demokratie</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>/dɪˈmɒkrəsi/</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>A system of government where citizens choose leaders through voting.</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Democracy gives people the right to vote.</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Many countries practice democracy today.</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/Special:FilePath/Urne_Ballot_box_république.jpg?width=400</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>2</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #9
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5572,8 +5572,59 @@
           <t>2026-04-19</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>furious</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>wütend</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>/ˈfjʊəriəs/</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Extremely angry or full of rage.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>She was furious when she discovered the broken window.</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>The coach became furious after the team lost the game.</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="n">
+        <v>2</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #11
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5614,7 +5614,6 @@
           <t>The coach became furious after the team lost the game.</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
       <c r="I89" t="n">
         <v>2</v>
       </c>
@@ -5623,8 +5622,59 @@
           <t>2026-04-19</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>to blackmail</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>erpressen</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>/ˈblækmeɪl/</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>To demand money or favors by threatening to reveal compromising information about someone.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>He tried to blackmail her with old photographs.</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>The criminal blackmailed the businessman for thousands of dollars.</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="n">
+        <v>2</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #12
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5664,7 +5664,6 @@
           <t>The criminal blackmailed the businessman for thousands of dollars.</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
       <c r="I90" t="n">
         <v>2</v>
       </c>
@@ -5673,8 +5672,59 @@
           <t>2026-04-19</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>infatuated</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>vernarrt</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>/ɪnˈfætʃueɪtɪd/</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Possessed with an intense but short-lived passion or admiration for someone</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>She became infatuated with her new colleague.</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>He was infatuated with the idea of becoming famous.</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="n">
+        <v>2</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #13
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5714,7 +5714,6 @@
           <t>He was infatuated with the idea of becoming famous.</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
       <c r="I91" t="n">
         <v>2</v>
       </c>
@@ -5723,8 +5722,59 @@
           <t>2026-04-19</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>abstinent</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>enthaltsam</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>/ˈæbstɪnənt/</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Practicing self-restraint, especially from alcohol or certain foods.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>He has been abstinent from alcohol for two years.</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>She follows an abstinent lifestyle for health reasons.</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="n">
+        <v>3</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #14
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5764,7 +5764,6 @@
           <t>She follows an abstinent lifestyle for health reasons.</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
       <c r="I92" t="n">
         <v>3</v>
       </c>
@@ -5773,8 +5772,59 @@
           <t>2026-04-19</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>persistent</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>beharrlich, ausdauernd</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>/pəˈsɪstənt/</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Continuing firmly despite difficulty or opposition</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>She was persistent in her efforts to learn English.</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>The persistent rain lasted for three days.</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="n">
+        <v>2</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #15
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5814,7 +5814,6 @@
           <t>The persistent rain lasted for three days.</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
       <c r="I93" t="n">
         <v>2</v>
       </c>
@@ -5823,8 +5822,59 @@
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>to steep tea</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Tee ziehen lassen</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>/tuː stiːp tiː/</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Phrase</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>To let tea leaves sit in hot water to release flavor and color.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>You should steep tea for about three to five minutes.</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>She steeped the tea in boiling water before serving it.</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="n">
+        <v>2</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #16
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5864,7 +5864,6 @@
           <t>She steeped the tea in boiling water before serving it.</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
       <c r="I94" t="n">
         <v>2</v>
       </c>
@@ -5873,8 +5872,59 @@
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Personally Identifiable Information (PII)</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>personenbezogene Daten</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>/ˈpɜːrsənəli aɪˈdentɪfaɪəbl ˌɪnfərˈmeɪʃən/</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Phrase</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Data that can identify a specific individual, such as name, address, or social security number.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Companies must protect PII to comply with privacy regulations.</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Never share your PII with untrusted websites or emails.</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="n">
+        <v>3</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #17
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5914,7 +5914,6 @@
           <t>Never share your PII with untrusted websites or emails.</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
       <c r="I95" t="n">
         <v>3</v>
       </c>
@@ -5923,8 +5922,59 @@
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>pointless</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>sinnlos</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>/ˈpɔɪntləs/</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Having no purpose, use, or likelihood of success.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>It's pointless to argue about it now.</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>The meeting was completely pointless.</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="n">
+        <v>2</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #18
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5964,7 +5964,6 @@
           <t>The meeting was completely pointless.</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
       <c r="I96" t="n">
         <v>2</v>
       </c>
@@ -5973,8 +5972,59 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>cheerful</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>fröhlich</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>/ˈtʃɪəfəl/</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Noticeably happy and optimistic in mood or manner.</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>She greeted us with a cheerful smile.</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>The children were cheerful despite the rain.</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="n">
+        <v>2</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #20
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6014,7 +6014,6 @@
           <t>The children were cheerful despite the rain.</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
       <c r="I97" t="n">
         <v>2</v>
       </c>
@@ -6023,8 +6022,59 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>clumsy</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>ungeschickt</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>/ˈklʌmzi/</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Moving or doing things in an awkward way, often causing accidents or mistakes.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>He is too clumsy to carry those fragile dishes.</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>She made a clumsy attempt to catch the ball.</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="n">
+        <v>2</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #21
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6064,7 +6064,6 @@
           <t>She made a clumsy attempt to catch the ball.</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
       <c r="I98" t="n">
         <v>2</v>
       </c>
@@ -6073,8 +6072,63 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>exploitation</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Ausbeutung</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>/ˌeksplɔɪˈteɪʃən/</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>The action of treating someone unfairly to benefit from their work or resources.</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>The exploitation of workers in factories was common during the industrial revolution.</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Environmental exploitation leads to the destruction of natural habitats.</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/Special:FilePath/Continental_AG_tire_factory_Mittellandkanal_Stoecken_Hannover_Germany_02.jpg?width=400</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>3</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #22
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6127,8 +6127,59 @@
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>invocable</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>aufrufbar</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>/ɪnˈvoʊkəbl/</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Capable of being called upon or summoned, especially in programming or legal contexts.</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>The function is invocable from any part of the code.</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>This right is invocable by any citizen under the law.</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="n">
+        <v>3</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #23
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6169,7 +6169,6 @@
           <t>This right is invocable by any citizen under the law.</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
       <c r="I100" t="n">
         <v>3</v>
       </c>
@@ -6178,8 +6177,63 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Pitfall</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Falle, Fallstrick</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>/ˈpɪtfɔːl/</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>A hidden or unexpected danger or difficulty.</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>One pitfall of online shopping is hidden delivery costs.</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Avoid the common pitfall of studying only the night before exams.</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/Special:FilePath/Insect_trap_hidden_in_a_tree_trunk_in_Junkerdalsura.jpg?width=400</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>2</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #24
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6232,8 +6232,59 @@
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>effortless</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>mühelos</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>/ˈefətləs/</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Requiring no physical or mental effort; done with ease.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>She made the difficult task look effortless.</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>His effortless style impressed everyone at the party.</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="n">
+        <v>2</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #26
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6274,7 +6274,6 @@
           <t>His effortless style impressed everyone at the party.</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
       <c r="I102" t="n">
         <v>2</v>
       </c>
@@ -6283,8 +6282,59 @@
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>to stack</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>stapeln</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>/stæk/</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>To arrange things in a neat pile, one on top of another.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Please stack the chairs after the meeting.</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>She stacked the books on the shelf.</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="n">
+        <v>1</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #27
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6324,7 +6324,6 @@
           <t>She stacked the books on the shelf.</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
       <c r="I103" t="n">
         <v>1</v>
       </c>
@@ -6333,8 +6332,59 @@
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>to sift</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>sieben</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>/sɪft/</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>To pass a substance through a sieve to remove lumps or separate particles.</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>She sifted the flour before making the cake.</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>They sifted through the evidence to find clues.</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="n">
+        <v>2</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #28
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6374,7 +6374,6 @@
           <t>They sifted through the evidence to find clues.</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
       <c r="I104" t="n">
         <v>2</v>
       </c>
@@ -6383,8 +6382,59 @@
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>to dissolve</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>auflösen</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>/dɪˈzɒlv/</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>To become or cause to become incorporated into a liquid so as to form a solution.</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Sugar dissolves quickly in hot water.</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>The tablet will dissolve in your mouth.</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="n">
+        <v>2</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #29
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6424,7 +6424,6 @@
           <t>The tablet will dissolve in your mouth.</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
       <c r="I105" t="n">
         <v>2</v>
       </c>
@@ -6433,8 +6432,59 @@
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>red tape</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Bürokratie</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>/red teɪp/</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Phrase</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Excessive bureaucracy or adherence to rules and formalities, especially in public business.</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>The company struggled with red tape when applying for permits.</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>We need to cut through the red tape to get this approved quickly.</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="n">
+        <v>2</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA-FIX: Bild fuer 'threshold' aktualisiert (Issue #31)
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -702,7 +702,11 @@
           <t>She stood at the threshold of the doorway, hesitating before stepping inside.</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/Special:FilePath/Funchal_(Madeira,_Portugal),_Rua_de_Santa_Maria_1_--_2025_--_0818.jpg?width=400</t>
+        </is>
+      </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
           <t>B2</t>
@@ -6474,7 +6478,6 @@
           <t>We need to cut through the red tape to get this approved quickly.</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
       <c r="I106" t="n">
         <v>2</v>
       </c>
@@ -6483,7 +6486,6 @@
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
           <t>Allgemein</t>

</xml_diff>

<commit_message>
ETA: Neues Wort 'distorted' aus Issue #33
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6487,6 +6487,58 @@
         </is>
       </c>
       <c r="L106" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>distorted</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>verzerrt</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>/dɪˈstɔːtɪd/</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Changed from the original shape, sound, or meaning in an unusual way.</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>The mirror showed a distorted reflection of my face.</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>The audio was distorted and hard to understand.</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="n">
+        <v>2</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort 'Retention' aus Issue #34
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6528,7 +6528,6 @@
           <t>The audio was distorted and hard to understand.</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
       <c r="I107" t="n">
         <v>2</v>
       </c>
@@ -6537,8 +6536,63 @@
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Retention</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Beibehaltung</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>/rɪˈtenʃən/</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>The continued possession, use, or control of something.</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Customer retention is crucial for business success.</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>The company improved employee retention through better benefits.</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/Special:FilePath/Mercy_Health_Partners_of_Southwest_Ohio_senior_health_and_housing_services_recruitment_and_retention_(R_&amp;_R)_initiative_-_DPLA_-_b80e071d7a1f9ae003c0c81c7ceacd77.jpg?width=400</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>2</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort 'pensive' aus Issue #35
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6591,8 +6591,59 @@
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>pensive</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>nachdenklich</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>/ˈpensɪv/</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Engaged in deep or serious thought, often with a hint of sadness.</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>She had a pensive look on her face.</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>He sat pensive by the window, thinking about his future.</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="n">
+        <v>2</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort 'blunt' aus Issue #36
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6633,7 +6633,6 @@
           <t>He sat pensive by the window, thinking about his future.</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
       <c r="I109" t="n">
         <v>2</v>
       </c>
@@ -6642,10 +6641,61 @@
           <t>2026-05-24</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
           <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>blunt</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>stumpf, direkt</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>/blʌnt/</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Not sharp or pointed; saying what you think without trying to be polite.</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>The knife was too blunt to cut the bread.</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>She was very blunt and told him the truth.</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="n">
+        <v>2</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>TV</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETA-FIX: Bild fuer 'tablecloth' aktualisiert (Issue #38)
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -5068,7 +5068,11 @@
           <t>The tablecloth is covered in wine stains — it needs a good wash.</t>
         </is>
       </c>
-      <c r="H79" s="5" t="inlineStr"/>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/Special:FilePath/Table-cloth_2008-1.jpg?width=400</t>
+        </is>
+      </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
           <t>A2</t>
@@ -6683,7 +6687,6 @@
           <t>She was very blunt and told him the truth.</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
       <c r="I110" t="n">
         <v>2</v>
       </c>
@@ -6692,7 +6695,6 @@
           <t>2026-05-24</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
           <t>TV</t>

</xml_diff>

<commit_message>
ETA: Neues Wort 'meanest' aus Issue #42
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fortschritt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fortschritt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L185"/>
+  <dimension ref="A1:L186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5454,7 +5454,6 @@
           <t>There is a significant difference between the two proposals.</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
         <is>
           <t>B1</t>
@@ -5465,7 +5464,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -5508,7 +5506,6 @@
           <t>He made a subtle hint that he wanted to leave early.</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
           <t>B2</t>
@@ -5519,7 +5516,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -5562,7 +5558,6 @@
           <t>He showed a genuine interest in learning the language.</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr">
         <is>
           <t>B1</t>
@@ -5573,7 +5568,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -5616,7 +5610,6 @@
           <t>The film's special effects were absolutely remarkable.</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
           <t>B1</t>
@@ -5627,7 +5620,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -5670,7 +5662,6 @@
           <t>It was considerate of her to send a thank-you note.</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr">
         <is>
           <t>B2</t>
@@ -5681,7 +5672,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -5724,7 +5714,6 @@
           <t>The persistent rain ruined our picnic plans.</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
           <t>B2</t>
@@ -5735,7 +5724,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -5778,7 +5766,6 @@
           <t>She felt anxious waiting for the doctor's call.</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
       <c r="I92" t="inlineStr">
         <is>
           <t>B1</t>
@@ -5789,7 +5776,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -5832,7 +5818,6 @@
           <t>He looked exhausted after working three back-to-back night shifts.</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
           <t>A2</t>
@@ -5843,7 +5828,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -5886,7 +5870,6 @@
           <t>She felt frustrated when nobody listened to her ideas.</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
       <c r="I94" t="inlineStr">
         <is>
           <t>A2</t>
@@ -5897,7 +5880,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -5940,7 +5922,6 @@
           <t>She felt deeply relieved when she passed the driving test.</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
           <t>B1</t>
@@ -5951,7 +5932,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -5994,7 +5974,6 @@
           <t>She felt awkward being the only person who didn't know anyone at the party.</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr">
         <is>
           <t>B1</t>
@@ -6005,7 +5984,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6048,7 +6026,6 @@
           <t>He is a decent person who always tries to do the right thing.</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
           <t>B1</t>
@@ -6059,7 +6036,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6102,7 +6078,6 @@
           <t>The documentary used vivid colours to bring the wildlife to life.</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr">
         <is>
           <t>B2</t>
@@ -6113,7 +6088,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6156,7 +6130,6 @@
           <t>She made a compelling argument for increasing the budget.</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
           <t>C1</t>
@@ -6167,7 +6140,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6210,7 +6182,6 @@
           <t>She was grateful that the rain stopped before the outdoor ceremony.</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr">
         <is>
           <t>A2</t>
@@ -6221,7 +6192,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6264,7 +6234,6 @@
           <t>After years in business, she had grown cynical about people's motives.</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
           <t>C1</t>
@@ -6275,7 +6244,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6318,7 +6286,6 @@
           <t>The investors took a cautious approach in the uncertain market.</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr">
         <is>
           <t>B1</t>
@@ -6329,7 +6296,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6372,7 +6338,6 @@
           <t>He was unhappy with his mediocre exam results.</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
           <t>B2</t>
@@ -6383,7 +6348,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6426,7 +6390,6 @@
           <t>He wore a bold red jacket that stood out in the crowd.</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
       <c r="I104" t="inlineStr">
         <is>
           <t>B1</t>
@@ -6437,7 +6400,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6480,7 +6442,6 @@
           <t>She felt an overwhelming sense of relief when the operation was over.</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
           <t>B2</t>
@@ -6491,7 +6452,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6534,7 +6494,6 @@
           <t>The team achieved great results despite limited resources.</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr">
         <is>
           <t>A2</t>
@@ -6545,7 +6504,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6588,7 +6546,6 @@
           <t>Animals adapt to their surroundings over thousands of years.</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
           <t>B1</t>
@@ -6599,7 +6556,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6642,7 +6598,6 @@
           <t>He didn't appreciate how hard she worked until she left.</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
       <c r="I108" t="inlineStr">
         <is>
           <t>B1</t>
@@ -6653,7 +6608,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6696,7 +6650,6 @@
           <t>I assumed he would be late, but he actually arrived early.</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
           <t>B1</t>
@@ -6707,7 +6660,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6750,7 +6702,6 @@
           <t>She avoided making eye contact during the difficult conversation.</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr">
         <is>
           <t>A2</t>
@@ -6761,7 +6712,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6804,7 +6754,6 @@
           <t>This role will challenge you in ways you have never experienced before.</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
           <t>B1</t>
@@ -6815,7 +6764,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6858,7 +6806,6 @@
           <t>I couldn't convince her that the film was worth watching.</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
       <c r="I112" t="inlineStr">
         <is>
           <t>B1</t>
@@ -6869,7 +6816,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6912,7 +6858,6 @@
           <t>Teaching demands a great deal of patience and dedication.</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
           <t>B1</t>
@@ -6923,7 +6868,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -6966,7 +6910,6 @@
           <t>She emphasized that the deadline was non-negotiable.</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr">
         <is>
           <t>B2</t>
@@ -6977,7 +6920,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7020,7 +6962,6 @@
           <t>The coach encouraged the team after a difficult first half.</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7031,7 +6972,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7074,7 +7014,6 @@
           <t>Don't hesitate to call me if you need any help.</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7085,7 +7024,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7128,7 +7066,6 @@
           <t>Social media can heavily influence the way young people see themselves.</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7139,7 +7076,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7182,7 +7118,6 @@
           <t>The union negotiated improved holiday allowances for all staff.</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
           <t>B2</t>
@@ -7193,7 +7128,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7236,7 +7170,6 @@
           <t>He worked hard to overcome the obstacles in his path.</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7247,7 +7180,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7290,7 +7222,6 @@
           <t>The police pursued the suspect through the city streets.</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr">
         <is>
           <t>B2</t>
@@ -7301,7 +7232,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7344,7 +7274,6 @@
           <t>The company was recognized for its outstanding customer service.</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
           <t>A2</t>
@@ -7355,7 +7284,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7398,7 +7326,6 @@
           <t>He relied on public transport to get to work every day.</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7409,7 +7336,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7452,7 +7378,6 @@
           <t>She finally revealed the secret she had been keeping for years.</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7463,7 +7388,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7506,7 +7430,6 @@
           <t>The police suspected the neighbour from the very beginning.</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7517,7 +7440,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7560,7 +7482,6 @@
           <t>We are witnessing a major shift in the way people communicate.</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
           <t>B2</t>
@@ -7571,7 +7492,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7614,7 +7534,6 @@
           <t>Learning a new language is a remarkable achievement at any age.</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7625,7 +7544,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7668,7 +7586,6 @@
           <t>Her calm approach to conflict made her an effective manager.</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7679,7 +7596,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7722,7 +7638,6 @@
           <t>They had a serious argument about money and didn't speak for a week.</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
       <c r="I128" t="inlineStr">
         <is>
           <t>A2</t>
@@ -7733,7 +7648,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7776,7 +7690,6 @@
           <t>You need to change your attitude if you want to succeed.</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7787,7 +7700,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7830,7 +7742,6 @@
           <t>The main challenge is keeping costs low while improving quality.</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
       <c r="I130" t="inlineStr">
         <is>
           <t>B1</t>
@@ -7841,7 +7752,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7884,7 +7794,6 @@
           <t>Under no circumstance should you share your password with anyone.</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
           <t>B2</t>
@@ -7895,7 +7804,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7938,7 +7846,6 @@
           <t>Marriage is a serious commitment that requires work from both partners.</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
       <c r="I132" t="inlineStr">
         <is>
           <t>B2</t>
@@ -7949,7 +7856,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K132" t="inlineStr"/>
       <c r="L132" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -7992,7 +7898,6 @@
           <t>She expressed concern about the rising cost of living.</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr">
         <is>
           <t>B1</t>
@@ -8003,7 +7908,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K133" t="inlineStr"/>
       <c r="L133" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8046,7 +7950,6 @@
           <t>The UN is working to resolve the conflict peacefully.</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
       <c r="I134" t="inlineStr">
         <is>
           <t>B1</t>
@@ -8057,7 +7960,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K134" t="inlineStr"/>
       <c r="L134" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8100,7 +8002,6 @@
           <t>We must consider the consequences of our decisions carefully.</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr">
         <is>
           <t>B2</t>
@@ -8111,7 +8012,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8154,7 +8054,6 @@
           <t>This word has a different meaning depending on the context.</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
       <c r="I136" t="inlineStr">
         <is>
           <t>B2</t>
@@ -8165,7 +8064,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8208,7 +8106,6 @@
           <t>The ethical dilemma had no easy answer.</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
           <t>B2</t>
@@ -8219,7 +8116,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8262,7 +8158,6 @@
           <t>There is growing evidence that exercise improves mental health.</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
       <c r="I138" t="inlineStr">
         <is>
           <t>B1</t>
@@ -8273,7 +8168,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8316,7 +8210,6 @@
           <t>The power failure left half the city without electricity.</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
           <t>B1</t>
@@ -8327,7 +8220,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K139" t="inlineStr"/>
       <c r="L139" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8370,7 +8262,6 @@
           <t>Smoking is a habit that is very difficult to break.</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
       <c r="I140" t="inlineStr">
         <is>
           <t>A2</t>
@@ -8381,7 +8272,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8424,7 +8314,6 @@
           <t>Climate change is having a devastating impact on coral reefs.</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
           <t>B1</t>
@@ -8435,7 +8324,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8478,7 +8366,6 @@
           <t>I have every intention of finishing this project on time.</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
       <c r="I142" t="inlineStr">
         <is>
           <t>B2</t>
@@ -8489,7 +8376,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K142" t="inlineStr"/>
       <c r="L142" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8532,7 +8418,6 @@
           <t>He seized every opportunity to practise his English.</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr">
         <is>
           <t>B1</t>
@@ -8543,7 +8428,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K143" t="inlineStr"/>
       <c r="L143" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8586,7 +8470,6 @@
           <t>It is important to consider the situation from different perspectives.</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
       <c r="I144" t="inlineStr">
         <is>
           <t>B2</t>
@@ -8597,7 +8480,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr"/>
       <c r="L144" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8640,7 +8522,6 @@
           <t>The government set education as its top priority for the coming year.</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr">
         <is>
           <t>B2</t>
@@ -8651,7 +8532,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8694,7 +8574,6 @@
           <t>She took full responsibility for the mistake and apologised publicly.</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
       <c r="I146" t="inlineStr">
         <is>
           <t>B1</t>
@@ -8705,7 +8584,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K146" t="inlineStr"/>
       <c r="L146" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8748,7 +8626,6 @@
           <t>They offered a reward for anyone who could find the lost dog.</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr">
         <is>
           <t>B1</t>
@@ -8759,7 +8636,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8802,7 +8678,6 @@
           <t>There is a risk of flooding in low-lying areas after heavy rain.</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
       <c r="I148" t="inlineStr">
         <is>
           <t>A2</t>
@@ -8813,7 +8688,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr"/>
       <c r="L148" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8856,7 +8730,6 @@
           <t>Talking it through calmly is often the best solution to an argument.</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
       <c r="I149" t="inlineStr">
         <is>
           <t>A2</t>
@@ -8867,7 +8740,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K149" t="inlineStr"/>
       <c r="L149" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8910,7 +8782,6 @@
           <t>Playing chess requires careful strategy and forward thinking.</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
       <c r="I150" t="inlineStr">
         <is>
           <t>B2</t>
@@ -8921,7 +8792,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -8964,7 +8834,6 @@
           <t>The documentary showed the daily struggle of people living in poverty.</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr"/>
       <c r="I151" t="inlineStr">
         <is>
           <t>B1</t>
@@ -8975,7 +8844,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K151" t="inlineStr"/>
       <c r="L151" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9018,7 +8886,6 @@
           <t>It took years to rebuild the trust after he had lied.</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
       <c r="I152" t="inlineStr">
         <is>
           <t>A2</t>
@@ -9029,7 +8896,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9072,7 +8938,6 @@
           <t>Living with uncertainty is a skill that requires practise and resilience.</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr"/>
       <c r="I153" t="inlineStr">
         <is>
           <t>B2</t>
@@ -9083,7 +8948,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9126,7 +8990,6 @@
           <t>Her awareness of other people's feelings made her an excellent therapist.</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr">
         <is>
           <t>B2</t>
@@ -9137,7 +9000,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K154" t="inlineStr"/>
       <c r="L154" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9180,7 +9042,6 @@
           <t>The film builds tension slowly before the shocking final scene.</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr">
         <is>
           <t>B1</t>
@@ -9191,7 +9052,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9234,7 +9094,6 @@
           <t>She finally figured out why the machine kept stopping.</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
       <c r="I156" t="inlineStr">
         <is>
           <t>B1</t>
@@ -9245,7 +9104,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K156" t="inlineStr"/>
       <c r="L156" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9288,7 +9146,6 @@
           <t>He gave up smoking after twenty years.</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr">
         <is>
           <t>A2</t>
@@ -9299,7 +9156,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K157" t="inlineStr"/>
       <c r="L157" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9342,7 +9198,6 @@
           <t>She looks forward to her morning coffee every single day.</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
       <c r="I158" t="inlineStr">
         <is>
           <t>A2</t>
@@ -9353,7 +9208,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K158" t="inlineStr"/>
       <c r="L158" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9396,7 +9250,6 @@
           <t>His creative approach made his application stand out from all the others.</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr">
         <is>
           <t>B1</t>
@@ -9407,7 +9260,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K159" t="inlineStr"/>
       <c r="L159" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9450,7 +9302,6 @@
           <t>Let's have coffee soon – I'd love to catch up with you.</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
       <c r="I160" t="inlineStr">
         <is>
           <t>B1</t>
@@ -9461,7 +9312,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K160" t="inlineStr"/>
       <c r="L160" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9504,7 +9354,6 @@
           <t>The constant noise was putting her off her work.</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr">
         <is>
           <t>B1</t>
@@ -9515,7 +9364,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K161" t="inlineStr"/>
       <c r="L161" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9558,7 +9406,6 @@
           <t>He came across as very confident during the interview.</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr">
         <is>
           <t>B2</t>
@@ -9569,7 +9416,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K162" t="inlineStr"/>
       <c r="L162" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9612,7 +9458,6 @@
           <t>I can't make up my mind – both options have their advantages.</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr"/>
       <c r="I163" t="inlineStr">
         <is>
           <t>B1</t>
@@ -9623,7 +9468,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K163" t="inlineStr"/>
       <c r="L163" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9666,7 +9510,6 @@
           <t>Please keep in mind that we have a limited budget for this project.</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
       <c r="I164" t="inlineStr">
         <is>
           <t>B1</t>
@@ -9677,7 +9520,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K164" t="inlineStr"/>
       <c r="L164" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9720,7 +9562,6 @@
           <t>He took his friends for granted until they were no longer around.</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr"/>
       <c r="I165" t="inlineStr">
         <is>
           <t>B2</t>
@@ -9731,7 +9572,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K165" t="inlineStr"/>
       <c r="L165" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9774,7 +9614,6 @@
           <t>The car ran out of petrol on the motorway.</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr">
         <is>
           <t>B1</t>
@@ -9785,7 +9624,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K166" t="inlineStr"/>
       <c r="L166" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9828,7 +9666,6 @@
           <t>Do you think the new flatmates will get along with each other?</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr"/>
       <c r="I167" t="inlineStr">
         <is>
           <t>B1</t>
@@ -9839,7 +9676,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K167" t="inlineStr"/>
       <c r="L167" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9882,7 +9718,6 @@
           <t>Can you point out the house on the map?</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr">
         <is>
           <t>B1</t>
@@ -9893,7 +9728,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K168" t="inlineStr"/>
       <c r="L168" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9936,7 +9770,6 @@
           <t>She was brought up by her grandparents in a small village.</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
           <t>B2</t>
@@ -9947,7 +9780,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K169" t="inlineStr"/>
       <c r="L169" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -9990,7 +9822,6 @@
           <t>They carried on working even when the power went out.</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr">
         <is>
           <t>A2</t>
@@ -10001,7 +9832,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K170" t="inlineStr"/>
       <c r="L170" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -10044,7 +9874,6 @@
           <t>The book kept me in suspense right until the final page.</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr">
         <is>
           <t>B1</t>
@@ -10055,7 +9884,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K171" t="inlineStr"/>
       <c r="L171" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10098,7 +9926,6 @@
           <t>The best plot twists make you want to rewatch the whole film.</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr">
         <is>
           <t>B1</t>
@@ -10109,7 +9936,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K172" t="inlineStr"/>
       <c r="L172" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10152,7 +9978,6 @@
           <t>Soap operas are famous for their dramatic cliffhangers.</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr">
         <is>
           <t>B2</t>
@@ -10163,7 +9988,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K173" t="inlineStr"/>
       <c r="L173" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10206,7 +10030,6 @@
           <t>We follow the protagonist on her journey from poverty to success.</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr">
         <is>
           <t>B2</t>
@@ -10217,7 +10040,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K174" t="inlineStr"/>
       <c r="L174" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10260,7 +10082,6 @@
           <t>A great story needs a compelling antagonist, not just a great hero.</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr"/>
       <c r="I175" t="inlineStr">
         <is>
           <t>C1</t>
@@ -10271,7 +10092,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K175" t="inlineStr"/>
       <c r="L175" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10314,7 +10134,6 @@
           <t>The film cuts to a flashback every time she hears that song.</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr">
         <is>
           <t>B1</t>
@@ -10325,7 +10144,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K176" t="inlineStr"/>
       <c r="L176" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10368,7 +10186,6 @@
           <t>Looking back, the foreshadowing was obvious – we just didn't notice it at first.</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr">
         <is>
           <t>C1</t>
@@ -10379,7 +10196,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K177" t="inlineStr"/>
       <c r="L177" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10422,7 +10238,6 @@
           <t>He accidentally gave away a major spoiler and everyone was furious.</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr">
         <is>
           <t>A2</t>
@@ -10433,7 +10248,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K178" t="inlineStr"/>
       <c r="L178" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10476,7 +10290,6 @@
           <t>She binge-watched three seasons of the show without leaving the sofa.</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr"/>
       <c r="I179" t="inlineStr">
         <is>
           <t>A2</t>
@@ -10487,7 +10300,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K179" t="inlineStr"/>
       <c r="L179" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10530,7 +10342,6 @@
           <t>She stayed up until 2 a.m. to watch the season finale live.</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr"/>
       <c r="I180" t="inlineStr">
         <is>
           <t>A2</t>
@@ -10541,7 +10352,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K180" t="inlineStr"/>
       <c r="L180" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10584,7 +10394,6 @@
           <t>A well-crafted subplot can be just as engaging as the main story.</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr"/>
       <c r="I181" t="inlineStr">
         <is>
           <t>C1</t>
@@ -10595,7 +10404,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K181" t="inlineStr"/>
       <c r="L181" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10638,7 +10446,6 @@
           <t>Critics praised the film for its exceptional character development.</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr"/>
       <c r="I182" t="inlineStr">
         <is>
           <t>B2</t>
@@ -10649,7 +10456,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K182" t="inlineStr"/>
       <c r="L182" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10692,7 +10498,6 @@
           <t>She used personal narrative to make her speech more engaging.</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr"/>
       <c r="I183" t="inlineStr">
         <is>
           <t>C1</t>
@@ -10703,7 +10508,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K183" t="inlineStr"/>
       <c r="L183" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10746,7 +10550,6 @@
           <t>The film blends the sci-fi and horror genres in a unique way.</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr"/>
       <c r="I184" t="inlineStr">
         <is>
           <t>B1</t>
@@ -10757,7 +10560,6 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K184" t="inlineStr"/>
       <c r="L184" t="inlineStr">
         <is>
           <t>TV</t>
@@ -10800,7 +10602,6 @@
           <t>The screenplay won an Oscar before the film was even shot.</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr"/>
       <c r="I185" t="inlineStr">
         <is>
           <t>B2</t>
@@ -10811,10 +10612,61 @@
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="K185" t="inlineStr"/>
       <c r="L185" t="inlineStr">
         <is>
           <t>TV</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>meanest</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>gemeinste, niederträchtigste</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>/ˈmiːnɪst/</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Superlative form of mean; most unkind or cruel</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>That was the meanest thing anyone has ever said to me.</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>He is the meanest person I have ever met.</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr"/>
+      <c r="I186" t="n">
+        <v>2</v>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETA: Neues Wort 'Lunatic' aus Issue #43
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L186"/>
+  <dimension ref="A1:L187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10654,7 +10654,6 @@
           <t>He is the meanest person I have ever met.</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
       <c r="I186" t="n">
         <v>2</v>
       </c>
@@ -10663,8 +10662,63 @@
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="K186" t="inlineStr"/>
       <c r="L186" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Lunatic</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Verrückter</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>/ˈluː.nə.tɪk/</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>A person who behaves in a foolish or crazy way.</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>He drives like a lunatic on the highway.</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Only a lunatic would swim in that freezing water.</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/Special:FilePath/Person_in_CrazyFrog_costume_(from_cropped_PublicTransport_CrazyFrog).jpg?width=400</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>2</v>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr"/>
+      <c r="L187" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort 'swanky' aus Issue #44
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L187"/>
+  <dimension ref="A1:L188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10717,8 +10717,59 @@
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="K187" t="inlineStr"/>
       <c r="L187" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>swanky</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>protzig, schick</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>/ˈswæŋki/</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Stylishly luxurious and expensive, often showing off wealth or status.</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>They had dinner at a swanky restaurant downtown.</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>He wore a swanky suit to the party.</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr"/>
+      <c r="I188" t="n">
+        <v>2</v>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr"/>
+      <c r="L188" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #45
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L188"/>
+  <dimension ref="A1:L189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10759,7 +10759,6 @@
           <t>He wore a swanky suit to the party.</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
       <c r="I188" t="n">
         <v>2</v>
       </c>
@@ -10768,8 +10767,63 @@
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="K188" t="inlineStr"/>
       <c r="L188" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Lighthouse</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Leuchtturm</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>/ˈlaɪthaʊs/</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>A tower with a bright light that guides ships at sea.</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>The lighthouse warned ships about the dangerous rocks.</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>We visited an old lighthouse by the coast.</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/a/a6/Aerial_photograph_60D_2012_05_13_8760_DxO_retusche.jpg</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>2</v>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="inlineStr">
         <is>
           <t>Allgemein</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #46
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L189"/>
+  <dimension ref="A1:L190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10822,10 +10822,65 @@
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="K189" t="inlineStr"/>
       <c r="L189" t="inlineStr">
         <is>
           <t>Allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Ferris wheel</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Riesenrad</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>/ˈferɪs wiːl/</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>A large rotating wheel with passenger cabins attached to its rim.</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>We rode the Ferris wheel at the carnival.</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>The Ferris wheel offers a great view of the city.</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/8/89/Ain_Dubai_View.jpg/1920px-Ain_Dubai_View.jpg</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>1</v>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr"/>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>TV</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #47
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L190"/>
+  <dimension ref="A1:L191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10877,8 +10877,59 @@
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="K190" t="inlineStr"/>
       <c r="L190" t="inlineStr">
+        <is>
+          <t>TV</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>to stall</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>verzögern</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>/stɔːl/</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>To delay or stop making progress intentionally</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Stop stalling and answer my question.</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>The car engine stalled at the traffic light.</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr"/>
+      <c r="I191" t="n">
+        <v>2</v>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr"/>
+      <c r="L191" t="inlineStr">
         <is>
           <t>TV</t>
         </is>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #48
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fortschritt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fortschritt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M291"/>
+  <dimension ref="A1:M292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17576,6 +17576,63 @@
       <c r="M291" t="inlineStr">
         <is>
           <t>Bring einen Reiseadapter für dein Handyladegerät mit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>to indulge</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>sich hingeben</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>/ɪnˈdʌldʒ/</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>To allow oneself to enjoy something pleasurable, especially excessively.</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>I like to indulge in chocolate cake on weekends.</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Parents should not indulge their children's every whim.</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr"/>
+      <c r="I292" t="n">
+        <v>2</v>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr"/>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>Ich gebe mich am Wochenende gerne Schokoladenkuchen hin.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #49
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M292"/>
+  <dimension ref="A1:M293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17615,7 +17615,6 @@
           <t>Parents should not indulge their children's every whim.</t>
         </is>
       </c>
-      <c r="H292" t="inlineStr"/>
       <c r="I292" t="n">
         <v>2</v>
       </c>
@@ -17624,7 +17623,6 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="K292" t="inlineStr"/>
       <c r="L292" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -17633,6 +17631,67 @@
       <c r="M292" t="inlineStr">
         <is>
           <t>Ich gebe mich am Wochenende gerne Schokoladenkuchen hin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Physiotherapist</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Physiotherapeut</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>/ˌfɪziəʊˈθerəpɪst/</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>A healthcare professional who treats injuries and movement problems through physical methods like exercise and massage.</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>The physiotherapist helped me recover from my knee injury.</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>She works as a physiotherapist at the local hospital.</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/8/8c/Physical_Therapists_at_work.jpg</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>2</v>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr"/>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>Der Physiotherapeut half mir, mich von meiner Knieverletzung zu erholen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #50
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M293"/>
+  <dimension ref="A1:M294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17683,7 +17683,6 @@
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="K293" t="inlineStr"/>
       <c r="L293" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -17692,6 +17691,63 @@
       <c r="M293" t="inlineStr">
         <is>
           <t>Der Physiotherapeut half mir, mich von meiner Knieverletzung zu erholen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>no casualties</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>keine Opfer</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>/nəʊ ˈkæʒuəltiz/</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Phrase</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>No people were killed or injured in an incident or accident.</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>The building collapsed, but fortunately there were no casualties.</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>The fire was quickly extinguished with no casualties reported.</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr"/>
+      <c r="I294" t="n">
+        <v>2</v>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr"/>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>TV</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>Das Gebäude stürzte ein, aber glücklicherweise gab es keine Opfer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #51
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M294"/>
+  <dimension ref="A1:M295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17730,7 +17730,6 @@
           <t>The fire was quickly extinguished with no casualties reported.</t>
         </is>
       </c>
-      <c r="H294" t="inlineStr"/>
       <c r="I294" t="n">
         <v>2</v>
       </c>
@@ -17739,7 +17738,6 @@
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="K294" t="inlineStr"/>
       <c r="L294" t="inlineStr">
         <is>
           <t>TV</t>
@@ -17748,6 +17746,63 @@
       <c r="M294" t="inlineStr">
         <is>
           <t>Das Gebäude stürzte ein, aber glücklicherweise gab es keine Opfer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Manslaughter</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Totschlag</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>/ˈmænˌslɔːtər/</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>The unlawful killing of a person without intent or premeditation.</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>He was convicted of manslaughter after the accident.</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>The jury had to decide between murder and manslaughter.</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr"/>
+      <c r="I295" t="n">
+        <v>3</v>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr"/>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>TV</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>Er wurde nach dem Unfall wegen Totschlags verurteilt.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #52
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M295"/>
+  <dimension ref="A1:M296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17785,7 +17785,6 @@
           <t>The jury had to decide between murder and manslaughter.</t>
         </is>
       </c>
-      <c r="H295" t="inlineStr"/>
       <c r="I295" t="n">
         <v>3</v>
       </c>
@@ -17794,7 +17793,6 @@
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="K295" t="inlineStr"/>
       <c r="L295" t="inlineStr">
         <is>
           <t>TV</t>
@@ -17803,6 +17801,63 @@
       <c r="M295" t="inlineStr">
         <is>
           <t>Er wurde nach dem Unfall wegen Totschlags verurteilt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>to lurk</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>lauern</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>/lɜːrk/</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>To wait hidden, ready to attack or appear suddenly.</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>A cat was lurking in the bushes.</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Someone is lurking outside our house.</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr"/>
+      <c r="I296" t="n">
+        <v>2</v>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr"/>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>Eine Katze lauerte in den Büschen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #53
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M296"/>
+  <dimension ref="A1:M297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17840,7 +17840,6 @@
           <t>Someone is lurking outside our house.</t>
         </is>
       </c>
-      <c r="H296" t="inlineStr"/>
       <c r="I296" t="n">
         <v>2</v>
       </c>
@@ -17849,7 +17848,6 @@
           <t>2026-07-26</t>
         </is>
       </c>
-      <c r="K296" t="inlineStr"/>
       <c r="L296" t="inlineStr">
         <is>
           <t>Allgemein</t>
@@ -17858,6 +17856,63 @@
       <c r="M296" t="inlineStr">
         <is>
           <t>Eine Katze lauerte in den Büschen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Wholesome</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>gesund, heilsam</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>/ˈhoʊlsəm/</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Adjektiv</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Good for your health or character; morally beneficial and pure.</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>She enjoys wholesome food like fresh vegetables and fruit.</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>The movie is wholesome entertainment for the whole family.</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr"/>
+      <c r="I297" t="n">
+        <v>2</v>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr"/>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>TV</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>Sie genießt gesunde Nahrung wie frisches Gemüse und Obst.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v3.0 Focus First: Bild-Fix, neuer Heute-Screen, Card-first-Training (P1-P4)
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fortschritt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fortschritt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17615,8 +17615,10 @@
           <t>Parents should not indulge their children's every whim.</t>
         </is>
       </c>
-      <c r="I292" t="n">
-        <v>2</v>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
       </c>
       <c r="J292" t="inlineStr">
         <is>
@@ -17675,8 +17677,10 @@
           <t>https://upload.wikimedia.org/wikipedia/commons/8/8c/Physical_Therapists_at_work.jpg</t>
         </is>
       </c>
-      <c r="I293" t="n">
-        <v>2</v>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
       </c>
       <c r="J293" t="inlineStr">
         <is>
@@ -17730,8 +17734,10 @@
           <t>The fire was quickly extinguished with no casualties reported.</t>
         </is>
       </c>
-      <c r="I294" t="n">
-        <v>2</v>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
       </c>
       <c r="J294" t="inlineStr">
         <is>
@@ -17785,8 +17791,10 @@
           <t>The jury had to decide between murder and manslaughter.</t>
         </is>
       </c>
-      <c r="I295" t="n">
-        <v>3</v>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
       </c>
       <c r="J295" t="inlineStr">
         <is>
@@ -17840,8 +17848,10 @@
           <t>Someone is lurking outside our house.</t>
         </is>
       </c>
-      <c r="I296" t="n">
-        <v>2</v>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
       </c>
       <c r="J296" t="inlineStr">
         <is>
@@ -17895,16 +17905,16 @@
           <t>The movie is wholesome entertainment for the whole family.</t>
         </is>
       </c>
-      <c r="H297" t="inlineStr"/>
-      <c r="I297" t="n">
-        <v>2</v>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
       </c>
       <c r="J297" t="inlineStr">
         <is>
           <t>2026-07-26</t>
         </is>
       </c>
-      <c r="K297" t="inlineStr"/>
       <c r="L297" t="inlineStr">
         <is>
           <t>TV</t>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #54
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fortschritt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fortschritt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M297"/>
+  <dimension ref="A1:M298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17923,6 +17923,69 @@
       <c r="M297" t="inlineStr">
         <is>
           <t>Sie genießt gesunde Nahrung wie frisches Gemüse und Obst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Ambush</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Hinterhalt</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>/ˈæmbʊʃ/</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>A surprise attack from a hidden position against an unsuspecting target.</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>The soldiers were caught in an ambush on the mountain road.</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>The rebels set up an ambush near the village entrance.</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/3/38/Embuscade_%28Guerre_de_Vend%C3%A9e%29_-_Evariste_Carpentier_%281%29-.jpg?utm_source=en.wikipedia.org&amp;utm_campaign=api&amp;utm_content=thumbnail_unscaled</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr"/>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>TV</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>Die Soldaten gerieten auf der Bergstraße in einen Hinterhalt.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #56
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M298"/>
+  <dimension ref="A1:M299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17977,7 +17977,6 @@
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="K298" t="inlineStr"/>
       <c r="L298" t="inlineStr">
         <is>
           <t>TV</t>
@@ -17986,6 +17985,65 @@
       <c r="M298" t="inlineStr">
         <is>
           <t>Die Soldaten gerieten auf der Bergstraße in einen Hinterhalt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>retrieval mission</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Bergungseinsatz</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>/rɪˈtriːvəl ˈmɪʃən/</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Phrase</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>An operation to recover or bring back something or someone from a location.</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>The team went on a retrieval mission to recover the lost equipment.</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>The astronauts completed a successful retrieval mission in space.</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr"/>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr"/>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>TV</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>Das Team startete einen Bergungseinsatz, um die verlorene Ausrüstung zu bergen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilder: feste Thumbnail-URLs in IMG_URLS aufgeloest
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Vokabeln" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
ETA: Neues Wort aus Issue #57
</commit_message>
<xml_diff>
--- a/vokabeln.xlsx
+++ b/vokabeln.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M296"/>
+  <dimension ref="A1:M297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18424,6 +18424,69 @@
         </is>
       </c>
     </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Taillight</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Rücklicht</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>/ˈteɪllaɪt/</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Nomen</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>A red light at the rear of a vehicle that indicates its presence.</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>The broken taillight made the car unsafe to drive at night.</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Police officers often stop vehicles with missing taillights.</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/5/59/Reisebus.Heck.jpg/330px-Reisebus.Heck.jpg?utm_source=en.wikipedia.org&amp;utm_campaign=api&amp;utm_content=thumbnail</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr"/>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>TV</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>Das kaputte Rücklicht machte das Auto unsicher für nächtliche Fahrten.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>